<commit_message>
Megit pull origin mainrge branch 'main' of https://github.com/ansforge/IG-document-core into htr-FHIR 027c99bcf6101f37a6d84b39c66a06315c4a4a0d
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-DestinatairePrevu.xlsx
+++ b/main/ig/StructureDefinition-DestinatairePrevu.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-19T09:31:54+00:00</t>
+    <t>2025-05-20T13:20:55+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -249,7 +249,7 @@
     <t>Base</t>
   </si>
   <si>
-    <t>DestinatairePrevu.Destinataire</t>
+    <t>DestinatairePrevu.destinataire</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PersonneStructure
@@ -561,8 +561,8 @@
   <dimension ref="A1:AJ3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="25.15625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="25.15625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="24.9453125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="24.9453125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -592,7 +592,7 @@
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="25.15625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="24.9453125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>

</xml_diff>